<commit_message>
further work on ESCO pre-processing chain: occupation similarity matrix, skills metadata.
</commit_message>
<xml_diff>
--- a/references/data/data_sources_overview.xlsx
+++ b/references/data/data_sources_overview.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10111"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/ETH/epg-work/04_jrc_green-skills-regional/03_data-analysis/re4gt/references/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Documents\Projects\04_jrc_green-skills-regional\03_data-analysis\re4gt\references\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{37F2C5FD-E486-8E4D-A6D1-944BBA6D1A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-11540" yWindow="-28800" windowWidth="51200" windowHeight="28800"/>
+    <workbookView xWindow="-11535" yWindow="-28800" windowWidth="51195" windowHeight="28800"/>
   </bookViews>
   <sheets>
     <sheet name="data_sources_overview" sheetId="1" r:id="rId1"/>
@@ -20,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="31">
   <si>
     <t>esco</t>
   </si>
@@ -58,13 +57,7 @@
     <t>KldB 2010</t>
   </si>
   <si>
-    <t>abbreviation</t>
-  </si>
-  <si>
     <t>name</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> link(s)</t>
   </si>
   <si>
     <t xml:space="preserve"> statement(s)/disclaimer(s)</t>
@@ -93,6 +86,49 @@
 https://statistik.arbeitsagentur.de/DE/Statischer-Content/Grundlagen/Klassifikationen/Klassifikation-der-Berufe/KldB2010/Systematik-Verzeichnisse/Generische-Publikationen/Systematisches-Verzeichnis-Berufsbenennung.xls?__blob=publicationFile&amp;v=7
 https://statistik.arbeitsagentur.de/DE/Statischer-Content/Grundlagen/Klassifikationen/Klassifikation-der-Berufe/KldB2010/Arbeitshilfen/Umsteigeschluessel/Generische-Publikation/Umsteigeschluessel-KldB2010-ISCO-08.xls?__blob=publicationFile&amp;v=5
 https://statistik.arbeitsagentur.de/DE/Statischer-Content/Grundlagen/Klassifikationen/Klassifikation-der-Berufe/KldB2010/Systematik-Verzeichnisse/Generische-Publikationen/BerufssektorenundSegmente.xls?__blob=publicationFile&amp;v=8</t>
+  </si>
+  <si>
+    <t>availability</t>
+  </si>
+  <si>
+    <t>public, open</t>
+  </si>
+  <si>
+    <t>public, upon application</t>
+  </si>
+  <si>
+    <t>private, upon request</t>
+  </si>
+  <si>
+    <t>ESCO Green Skills Metadata</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> link(s), description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Training data set for labelling green skills and scores assigned by classifier
+As we agreed in our call the past week, please find attached one excel document including the following information:
+• Training set: exact list of data employed to train the classifier
+• Score: the score assigned by the classifier to every ESCO skill that is now labelled as green.
+Few considerations on the scores:
+• 5 skills have the text “Expert-driven” instead of the score. These are transversal skills that were still under review when we were finalising our classifier and were labelled as green by experts. We did not need the score in these cases.
+• Some skills have a low score compared the average. These are skills that were not considered as green by the classifier (below the threshold we set), but that were labelled as green in the human labelling activity. These have been reviewed and considered as green. 
+• [general rule] The preferred terms may have been subject to changes. I recommend using the URI when comparing different datasets.
+• In general, please consider the argumentation we discussed in our call. The classifier tells us how semantically close ESCO skills are to the green skills in the training dataset, and not what is their real impact on the environment.
+We kindly ask you not to share this information. If you know someone who is interested in this document, we would be happy to schedule a call and evaluate whether to share it.
+</t>
+  </si>
+  <si>
+    <t>04.03.2022 (shared by ESCO Team)</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>GreenLabellingData.xlsx</t>
+  </si>
+  <si>
+    <t>abbreviation/file/variable</t>
   </si>
 </sst>
 </file>
@@ -585,7 +621,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -601,6 +637,9 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -958,81 +997,91 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="85.5" style="1" customWidth="1"/>
-    <col min="4" max="4" width="58.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="82.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="10.83203125" style="1"/>
+    <col min="3" max="3" width="21.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="85.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="58.375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="82.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="10.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>15</v>
-      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>4</v>
@@ -1040,57 +1089,92 @@
       <c r="E4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>18</v>
+      <c r="F4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
+      <c r="C5" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
+      <c r="C6" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
+      <c r="C7" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
     </row>
-    <row r="8" spans="1:6" ht="388" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" ht="315" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="4">
+      <c r="E8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="4">
         <v>44610</v>
       </c>
-      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+    </row>
+    <row r="9" spans="1:7" ht="362.25" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>28</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
added new ds ref to list (esco brown skills). added functions for reading brown esco skill labels and creating a skill-based GBN classification. now we can compare the onet- and esco-based binary classifications quantitatively. assuming there will be a big difference, which makes for interesting insights!
</commit_message>
<xml_diff>
--- a/references/data/data_sources_overview.xlsx
+++ b/references/data/data_sources_overview.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="34">
   <si>
     <t>esco</t>
   </si>
@@ -129,6 +129,17 @@
   </si>
   <si>
     <t>abbreviation/file/variable</t>
+  </si>
+  <si>
+    <t>ESCO Brown Skills Metadata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In the meantime, please find attached the list of skills labelled as brown by one of our classifiers. As you may notice, the number of brown ESCO skills is limited compared to the overall dataset size. In fact, while we have trained our model on the three separate training sets (brown, white, green), the model we opted for to distinguish green skills is one that distinguishes between brown+white versus green. I can explain more in our call. 
+On our side, we would be very interested in the results of your manual validation. We would also be glad to learn more in case you are planning a similar work for other skill types – e.g. digital skills.
+</t>
+  </si>
+  <si>
+    <t>/</t>
   </si>
 </sst>
 </file>
@@ -621,7 +632,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -640,6 +651,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -997,7 +1011,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" style="1" bestFit="1" customWidth="1"/>
@@ -1169,10 +1183,36 @@
       <c r="D9" s="6" t="s">
         <v>26</v>
       </c>
+      <c r="E9" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="F9" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G9" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="141.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="7">
+        <v>44635</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>28</v>
       </c>
     </row>

</xml_diff>

<commit_message>
restructured data classes. implemented aggregation by isco occupation. added new data sources to references list.
</commit_message>
<xml_diff>
--- a/references/data/data_sources_overview.xlsx
+++ b/references/data/data_sources_overview.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="48">
   <si>
     <t>esco</t>
   </si>
@@ -140,6 +140,67 @@
   </si>
   <si>
     <t>/</t>
+  </si>
+  <si>
+    <t>ESCO-Zuordnungen.xlsx</t>
+  </si>
+  <si>
+    <t>public</t>
+  </si>
+  <si>
+    <t>contact</t>
+  </si>
+  <si>
+    <t>IT_mapping_23.04.2021.csv</t>
+  </si>
+  <si>
+    <t>mapping_ESCO-Berufenet_draft_20220324.csv</t>
+  </si>
+  <si>
+    <t>ESCO - IT Mapping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Christine.Vigeant@iab.de </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lieber Herr Zausinger,
+herzlichen Dank für Ihre Anfrage. Bitte entschuldigen Sie die verzögerte Antwort. 
+Der BW-Verlag hat vor ca. 2 Jahren umfangreiche Mappingtabellen erstellt, die auch in der DKZ-Recherche abrufbar sind. Sie können diese Listen im DKZ Download-Portal (https://download-portal.arbeitsagentur.de/files/start) herunterladen, das auch für Externe zugänglich ist. Die aktuelle Liste füge ich Ihnen bei.
+Wir hoffen, das hilft Ihnen etwas weiter. Bei Rückfragen können Sie sich gerne wieder an uns wenden.
+Viele Grüße
+Christine Vigeant
+Institut für Arbeitsmarkt- und Berufsforschung (IAB) 
+Presse- und Öffentlichkeitsarbeit 
+Regensburger Straße 100
+90478 Nürnberg 
+Tel.: 0911/177-2065
+E-Mail: Christine.Vigeant@iab.de 
+http://www.iab.de 
+</t>
+  </si>
+  <si>
+    <t>https://download-portal.arbeitsagentur.de/files/start</t>
+  </si>
+  <si>
+    <t>Mapping Tabellen DE: ESCO occupations - DE occupations (DKZ?), ESCO Skills - DE Kompetenzen</t>
+  </si>
+  <si>
+    <t>Mapping ESCO - DE (Berufenet)</t>
+  </si>
+  <si>
+    <t>public, currently undisclosed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dear Felix and Florian,
+Please find attached the mapping tables that connect the ESCO classification to the German and Italian classifications of occupations. I remind you that while the Italian mapping is complete, the German mapping must still be considered as a draft.
+These mappings have been done in the context of the EURES legislation – in the last call you seemed familiar with it. Officers from every Member State had the option to map using their own tools, or via the ESCO Mapping Platform. The mapping between two occupations is based on four labels, and you can read more here. The Italian colleagues also published this paper based on the mapping exercise.
+Hope you will find it useful! May you need any further assistance, please do not hesitate to contact us.
+Kind regards,
+Chiara
+</t>
+  </si>
+  <si>
+    <t>Chiara Stramaccioni &lt;chiara.stramaccioni@esco-support.eu&gt;</t>
   </si>
 </sst>
 </file>
@@ -632,7 +693,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -653,6 +714,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -1011,43 +1081,46 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.5" style="1" customWidth="1"/>
-    <col min="4" max="4" width="85.5" style="1" customWidth="1"/>
-    <col min="5" max="5" width="58.375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13.875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="82.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="10.875" style="1"/>
+    <col min="3" max="4" width="21.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="85.5" style="1" customWidth="1"/>
+    <col min="6" max="6" width="58.375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="13.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="82.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="10.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:8" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1055,20 +1128,21 @@
       <c r="C2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="2"/>
+      <c r="E2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -1076,20 +1150,21 @@
       <c r="C3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>4</v>
-      </c>
+      <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -1097,20 +1172,21 @@
       <c r="C4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>4</v>
-      </c>
+      <c r="D4" s="2"/>
       <c r="E4" s="2" t="s">
         <v>4</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -1122,8 +1198,9 @@
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
@@ -1135,8 +1212,9 @@
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -1148,8 +1226,9 @@
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:7" ht="315" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="315" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
@@ -1159,18 +1238,19 @@
       <c r="C8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="2"/>
+      <c r="E8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="4">
+      <c r="G8" s="4">
         <v>44610</v>
       </c>
-      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:7" ht="362.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="362.25" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>29</v>
       </c>
@@ -1180,20 +1260,20 @@
       <c r="C9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="141.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="141.75" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>29</v>
       </c>
@@ -1203,20 +1283,97 @@
       <c r="C10" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="E10" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F10" s="7">
+      <c r="G10" s="7">
         <v>44635</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="H10" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="267.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G11" s="7">
+        <v>44644</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="267.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G12" s="7">
+        <v>44644</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="362.25" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="G13" s="7">
+        <v>44645</v>
+      </c>
+      <c r="H13" s="1" t="s">
         <v>28</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D13" r:id="rId1"/>
+    <hyperlink ref="F13" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fixed bugs in eulfs preprocessing pipeline.
</commit_message>
<xml_diff>
--- a/references/data/data_sources_overview.xlsx
+++ b/references/data/data_sources_overview.xlsx
@@ -160,7 +160,28 @@
     <t>ESCO - IT Mapping</t>
   </si>
   <si>
-    <t xml:space="preserve">Christine.Vigeant@iab.de </t>
+    <t>https://download-portal.arbeitsagentur.de/files/start</t>
+  </si>
+  <si>
+    <t>Mapping Tabellen DE: ESCO occupations - DE occupations (DKZ?), ESCO Skills - DE Kompetenzen</t>
+  </si>
+  <si>
+    <t>Mapping ESCO - DE (Berufenet)</t>
+  </si>
+  <si>
+    <t>public, currently undisclosed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dear Felix and Florian,
+Please find attached the mapping tables that connect the ESCO classification to the German and Italian classifications of occupations. I remind you that while the Italian mapping is complete, the German mapping must still be considered as a draft.
+These mappings have been done in the context of the EURES legislation – in the last call you seemed familiar with it. Officers from every Member State had the option to map using their own tools, or via the ESCO Mapping Platform. The mapping between two occupations is based on four labels, and you can read more here. The Italian colleagues also published this paper based on the mapping exercise.
+Hope you will find it useful! May you need any further assistance, please do not hesitate to contact us.
+Kind regards,
+Chiara
+</t>
+  </si>
+  <si>
+    <t>Chiara Stramaccioni &lt;chiara.stramaccioni@esco-support.eu&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">Lieber Herr Zausinger,
@@ -175,32 +196,20 @@
 90478 Nürnberg 
 Tel.: 0911/177-2065
 E-Mail: Christine.Vigeant@iab.de 
-http://www.iab.de 
+http://www.iab.de
+Jana Bart (20.03.2022): DKZ ist eine interne ID für Einzelberufe in der Bundesagentur für Arbeit. Mit der Kompetenz ID werden die verschiedenen Arten von Kompetenzen klassifiziert in der BA. Sie brauchen nur die Codenummer, in der der 5-Steller der Kldb2010 steckt.
+Beispiel: Codenr B 11302-102  ---&gt;11302 ist der 5-Steller Kldb2010.
 </t>
   </si>
   <si>
-    <t>https://download-portal.arbeitsagentur.de/files/start</t>
-  </si>
-  <si>
-    <t>Mapping Tabellen DE: ESCO occupations - DE occupations (DKZ?), ESCO Skills - DE Kompetenzen</t>
-  </si>
-  <si>
-    <t>Mapping ESCO - DE (Berufenet)</t>
-  </si>
-  <si>
-    <t>public, currently undisclosed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dear Felix and Florian,
-Please find attached the mapping tables that connect the ESCO classification to the German and Italian classifications of occupations. I remind you that while the Italian mapping is complete, the German mapping must still be considered as a draft.
-These mappings have been done in the context of the EURES legislation – in the last call you seemed familiar with it. Officers from every Member State had the option to map using their own tools, or via the ESCO Mapping Platform. The mapping between two occupations is based on four labels, and you can read more here. The Italian colleagues also published this paper based on the mapping exercise.
-Hope you will find it useful! May you need any further assistance, please do not hesitate to contact us.
-Kind regards,
-Chiara
-</t>
-  </si>
-  <si>
-    <t>Chiara Stramaccioni &lt;chiara.stramaccioni@esco-support.eu&gt;</t>
+    <t>Christine.Vigeant@iab.de 
+Institut für Arbeitsmarkt- und Berufsforschung (IAB) 
+Presse- und Öffentlichkeitsarbeit 
+Regensburger Straße 100
+90478 Nürnberg 
+Tel.: 0911/177-2065
+E-Mail: Christine.Vigeant@iab.de 
+http://www.iab.de</t>
   </si>
 </sst>
 </file>
@@ -693,7 +702,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -724,6 +733,9 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -1304,13 +1316,13 @@
         <v>39</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>47</v>
-      </c>
       <c r="E11" s="6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G11" s="7">
         <v>44644</v>
@@ -1324,16 +1336,16 @@
         <v>38</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E12" s="6" t="s">
         <v>44</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>46</v>
       </c>
       <c r="G12" s="7">
         <v>44644</v>
@@ -1342,24 +1354,24 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="362.25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="F13" s="10" t="s">
         <v>40</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>42</v>
       </c>
       <c r="G13" s="7">
         <v>44645</v>
@@ -1370,7 +1382,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D13" r:id="rId1"/>
+    <hyperlink ref="D13" r:id="rId1" display="Christine.Vigeant@iab.de "/>
     <hyperlink ref="F13" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
added R scripts. extended gitignore to ignore R metadata files.
</commit_message>
<xml_diff>
--- a/references/data/data_sources_overview.xlsx
+++ b/references/data/data_sources_overview.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="53">
   <si>
     <t>esco</t>
   </si>
@@ -210,6 +210,54 @@
 Tel.: 0911/177-2065
 E-Mail: Christine.Vigeant@iab.de 
 http://www.iab.de</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lieber Herr Zaussinger,
+anbei sende ich Ihnen schon einmal das Datenstrukturfile (DSF). Ich schicke das im SPSS-Format. Meiner Erfahrung nach lassen sich SPSS- und stata-Formate gut über R einlesen. Bitte lassen Sie mich wissen, wenn Sie die Daten in anderer Form bekommen möchten. Die Daten für den GWAP und die KDFV werde ich nach Abschluss der Abstimmung in gleicher Form an den Standort Bayern übermitteln.
+Bitte beachten Sie:
+Was ist ein Datenstrukturfile?
+•             Ein Datenstrukturfile stellt ein Abbild der Originalmerkmale in Form einer sehr kleinen Stichprobe dar. Es beinhaltet jedoch nicht die Originaldaten!
+•             Durch technische Verfahren sind die Daten im Datenstrukturfile so verfälscht, dass nur noch synthetische, nicht sinnvoll interpretierbare Datensätze enthalten sind. 
+Was kann ein Datenstrukturfile leisten?
++             Das Datenstrukturfile ist eine Arbeitshilfe. Es dient der Entwicklung lauffähiger Analyseprogramme (Do-File, Programmcode, Syntax).
++             Es umfasst nicht alle beantragten Merkmale, die in den Originaldaten enthalten sind. Zur Orientierung nutzen Sie bitte das Schlüsselverzeichnis oder Ihren persönlich abgestimmten Merkmalskranz. 
++             Alle für Ihre Programmierung notwendigen Datensatzinformationen, die auch für die Originaldaten gelten, sind im Datenstrukturfile enthalten (z.B. Variablenlabels, Variablentypen und Formate, Wertelabels, Satzstellen). 
+Was sind die Grenzen eines Datenstrukturfiles?
+-              Das Datenstrukturfile bietet keine Datengrundlage für inhaltlich valide Aussagen. 
+-              Die Ausprägungen und Abhängigkeitsstrukturen zwischen Merkmalen im Datenstrukturfile entsprechen nicht denen der Originaldaten. Zusätzlich können Ausprägungen aufgrund der kleinen Stichprobe ggf. nicht belegt sein, die in den Originaldaten aber evtl. doch vorhanden sind. 
+-              Die mit dem Datenstrukturfile erzeugten Ergebnisse liefern keinen Hinweis, ob inhaltliche Fragestellungen adäquat umgesetzt werden können. 
+-              Aufgrund der kleinen Stichprobe des Datenstrukturfiles ist die Programmlaufzeit auf dem Datenstrukturfile um ein Vielfaches geringer als die Laufzeiten auf dem Originaldatensatz. 
+Bei Fragen wenden Sie sich bitte an Ihren zuständigen FDZ-Standort.
+Folgende Variablen sind anders als in den On-Site-Daten (KDFV und GWAP) nicht im DSF enthalten:
+EF196 EF196U3 EF196A EF196AU3 EF560UG1 EF560UG2 EF560U3 EF560U4 EF563 EF566 EF568 EF591 EF592 EF593 EF594 EF599 EF601 EF604
+Mit freundlichen Grüßen
+Im Auftrag
+gez. Colin Schmidt
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Information und Technik
+Nordrhein-Westfalen (IT.NRW)
+Statistisches Landesamt
+Postanschrift: Postfach 10 11 05 * 40002 Düsseldorf
+Dienstgebäude: Roßstraße 64 * 40476 Düsseldorf
+http://www.it.nrw.de
+S1 * Servicebündel Veröffentlichung * Forschungsdatenzentrum
+Forschungsdatenzentrum
+Tel.  +49211-9449-2939 * Fax +49211-9449-8087
+mailto:Colin.Schmidt@it.nrw.de
+mailto:forschungsdatenzentrum@it.nrw.de
+http://www.forschungsdatenzentrum.de
+</t>
+  </si>
+  <si>
+    <t>public, paid</t>
+  </si>
+  <si>
+    <t>Datenstrukturfile (DSF) Mikrozensus 2019</t>
+  </si>
+  <si>
+    <t>re4gt\data\raw\lfs\de\DSF_MZ 2019.CSV</t>
   </si>
 </sst>
 </file>
@@ -1093,7 +1141,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" style="1" bestFit="1" customWidth="1"/>
@@ -1380,6 +1428,23 @@
         <v>28</v>
       </c>
     </row>
+    <row r="14" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D13" r:id="rId1" display="Christine.Vigeant@iab.de "/>

</xml_diff>